<commit_message>
Updated CST6000_StudentList with 1st marking and comments
</commit_message>
<xml_diff>
--- a/CST6000_StudentList.xlsx
+++ b/CST6000_StudentList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CARDIFFMET\TEACHING 25-26\2025_26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025_26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB28F8C-078F-4EA3-B515-3B0D0AA0F580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60BF94BE-B255-4EA8-BDDF-85F8A768DA4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="82440" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B0E4C297-D52A-4FF0-90FD-99DCC2F2FD99}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B0E4C297-D52A-4FF0-90FD-99DCC2F2FD99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
   <si>
     <t xml:space="preserve">Name </t>
   </si>
@@ -108,13 +108,81 @@
   </si>
   <si>
     <t>st20233361@outlook.cardiffmet.ac.uk</t>
+  </si>
+  <si>
+    <t>1st Marker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2nd Marker </t>
+  </si>
+  <si>
+    <t>Agreed Y/N</t>
+  </si>
+  <si>
+    <t>Agreed Mark</t>
+  </si>
+  <si>
+    <t>First Marker Comments/Feedback</t>
+  </si>
+  <si>
+    <t>Your references are also listed in your Contents page and you have a jarring shift in font and text size in the Abstract. It is important to proof read your work prior to submission. 
+You make a few statements in your Introduction that I feel really do beg for support through research or further explanation. You state that 'modern' video games depend on user interfaces. So, what constitutes a 'modern' video game and haven't video games always utilised UI for this purpose? Pac-Man displays the number of lives the player has, their high score... It seems to be that you are inferring through omission that early video games didn't utilise UI, but they really did! I would have liked to have seen more evidence of research here. You don't really provide a very strong, evidence-based, rationale for what you are doing. It does improve in clarity as it continues through 2.2, 2.3 and 3.
+Your Literature Review is meant to be exactly that - a review of the existing literature in and around your field of interest, but where is the research? You seem to have condensed the research you have done into one part of the Lit Review (4.8) and that's it! There are numerous areas where you make statements or define terms that needed to be supported by academic literature (for example, the first paragraph of 4.1 there at least six points where it would have been appropriate to cite sources). It is also quite confusing, as you reference an outcome of the project in 4.4, but the project won't exist yet for the reader. The Literature Review is supposed to be the research that you do in order to understand what you will need to create, not to try to support what you already have created. 
+Not all HUDS are created equally - Your Lit Review would have been a good place to have an informed discussion on UI design in video games, where you could have introduced research around how quickly we look around the screen, why in Western games it is more likely that important HUD elements are in a top or bottom left corner. Colour schemes, font... there was so much that you could have included here that would have provided an evidence-based design for your artifact.
+Methodology - How were the participants selected? This would be important to know in case of bias. You do a good job here, but your ethics section (8) should have been included here too, and it's missing a few important points. How did you screen for participants? Was there anything that created an 'ideal' participant for this study and the data you were looking to collect? Did your questions align with the 2010 Equalities Act and respect protected characteristics? Were participants notified that there would be blood splatter before they began? Is reducing playtime an accepted way to counter this? If so, where is the research that supports this?
+Artifact Development - Was the choice only between Unity and Unreal? Do no other game engines exist? Did the artifact need to be 3D? It feels like the choice of game engine and style of game were decided beforehand, rather than researched, discussed and then decided upon. Again, as with the other sections, this section suffers from a lack of research. A lot of what is discussed here is relevant to the artifact, but it lacks an informed discussion as to why you would do X over Y. You have opted for a 'simple' health bar but not investigated other Action/FPS games to compare their HUDS. There is nothing here to inform the reader as to what a Basic UI looks like and what it has to contain to satisfy your Aims and Objectives. No UML?
+Your results are well discussed and key points identified with regard to the design and the experience of the participant. You have potentially identified that despite the 'Basic' design being more readable, that did not necessarily translate to it being a more enjoyable experience for the participant. I think that the issue with a lack of crosshair, confusion over the fire-button, and other reported issues could have been identified earlier and maybe indicates a lack of time spent planning and designing the artifact. 
+Overall there is some good work here, Garyn, and the latter part is definitely stronger than the first part. Where your project really felt lacking was the research. At L6 you should be used to gathering a lot of research and understanding why it is important to support statements and arguments with academic sources. Here it felt like more of an afterthought, and it really affected the credibility of what you were trying to do here. I wish you had booked more supervision time and gone over what you were doing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstract could have been longer and more detailed - It really covers the beginning and end with no focus on the methodology.
+Introduction - 'Mihaly Csikszentmihalyi states that games are enjoyed by allowing you the opportunity to go beyond the boundaries of 
+ordinary experience (Csikszentmihalyi 2002).' Is this a direct quote? If so you need to use quotation marks. As you are already mentioning the author in the sentence, you don't need to cite them again at the end, you just need to include the year after their name 'Mihaly Csikszentmihalyi (2002) states that...'. Where did that citation come from? There is no matching reference for it and Csikszentmihalyi's original work was in the mid-70s. If you are citing him via a later source you need to use secondary referencing. 
+If immersion has been a 'hot topic of discussion' then where is the evidence of this? If you make a statement or assertion then you need to support it with research. Watch you academic writing - 'do not' not 'don't' We do not use contractions.
+A good go at the Literature Review, and there is some good discussion here. I felt it needed more time and attention, and more research added. The focus of it seemed to drift, particularly as you are looking at light sources rather than other forms of navigation. It is fine to acknowledge they exist and to have a small discussion around them, but I would have expected to see a greater portion of that balance on lighting as navigation. Your citations are a little off in their formatting, and there are places where you mention a book without capitalisation or appropriate citation.
+Research Methodology - Again, citations! The 2010 Equality Act should be capitalised and it needs to be cited and referenced. This section is rather thin, with no discussion of ethics, apart from a nod to the 2010 Equality Act, but not specifically which parts of it are not needed or appropriate for the study, or what form the artefact will take and whether any aspect of it could negatively impact a participant. There needed to be a greater discussion here around potential issues, if only to negate them.
+Artifact - What is the rationale behind the design? Why a medieval castle? I would have expected some research and discussion over why this would be an objectively more immersive experience than another interior? Especially as you may have different types of light source, but the type and colour of light they emit is going to be largely similar. It could be argued that in a more modern interior, you could have introduced different colour lighting. If it was important to have the same colour lighting, then that is something to discuss. You seem to have pulled the castle design out of nowhere and decided that would be 'more immersive' without providing any rationale for it. Does the design of the interior, the aesthetics, actually matter as far as what you are seeking to test?
+'There has been research that shows players have bias to certain sides when navigating and taking in visual information in video games.' You are acknowledging that the research exists... so where is it? Sources?
+Have you defined what immersion is in this context? You state that it has been achieved through two main factors - models and lighting, but how do you know that those are two main factors? How are you defining 'modern' and 'older' games - examples would have helped here. 'Morrowind' was made around 25 years ago and that had an enormous map and lighting. Is exploration a result of advancing hardware techniques or an aspect of a particular game genre? Is exploration in a game uniquely tied to lighting? If there are links then you need to evidence them.
+Despite the lack of rationale behind the artifact, the testing is comprehensive with a sound approach to optimisation and bug fixing.
+Conclusion is fairly broad, largely because more needed to be done earlier to explore and identify immersion and exactly where the issue you were looking to address existed. You did not highlight any games where lighting had been an issue with regard to navigation. '...in which this research suggests many modern games are not using it optimally, this however will depend on the purpose of the game.' I would say it absolutely depends on the purpose of the game. This could be perhaps investigated more rigorously through selecting a specific genre of game to examine. Not all games are going to be needing to use light as a source of exploration or navigation. 'Phasmophobia' places an enormous importance on lighting in the game, but not for navigation.
+There is some good work here, Geraint. I feel you ran with the artefact before really getting into the research, and there were areas that you later drew on (such as immersion) that you had not explored satisfactorily. The testing is good. You have made some errors in your citation and referencing that I would not expect at L6 - particularly your reference section not being alphabetical by author. </t>
+  </si>
+  <si>
+    <t>Deferred</t>
+  </si>
+  <si>
+    <t>Exited</t>
+  </si>
+  <si>
+    <t>NS</t>
+  </si>
+  <si>
+    <t>Archchaya Jenganathan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No Abstract present. 
+The Introduction lacks clarity on the problem being addressed. There are a lot of travel apps (and for what form of transport, country...?) I did warn you in the single meeting we had that your project scope was too big and you needed to refine it. You have started without providing any evidence to support the problem you are trying to address or why those features would be important to have in a travel app, particularly as the term 'Travel App' sounds very vague and generic and it would need to be able to communicate with other systems to be effective, particularly in the UK. You state that there is a growing demand for this kind of app, but where is the evidence? 
+You have a Literature Review with no literature being reviewed? Where are your citations and references? You need to be engaging with the research and discussing it here. This is where you are supposed to be exploring the field (travel apps) and discussing what is out there, identifying the gaps in the market, and showing your understanding of these systems.  'This section critically reviews existing research on travel planning systems...' No it doesn't. You have not critically engaged with any research, which is not acceptable for a L6 research project.
+You started by saying that AI integration is a key feature, but then you later say that your AI-Based features are actually simulating AI behaviour. Is this not misrepresenting what the app does? How would you be explaining the ethics of that (the ethics of using Gen-AI, the plagiarism, the potential for inaccuracy aside) to a potential user of the app who may have chosen it based on it flaunted AI capabilities?
+The submitted project seems to be largely Python-based, but this wasn't mentioned. Only HTML, CSS and JavaScript.
+I really wish you had booked more meetings with me, Archchaya. I have no idea how you managed to do an L6 dissertation project without considering the necessity for research. It feels like you started with the artifact and then did everything around it to justify doing it, rather than leading with research in order to investigate what you needed to create. Without doing the research how can you successfully identify a gap or a problem? How can you evidence that it actually is a problem and not something that you believe to be a problem? The lack of engagement with any research really let you down here. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstract - Good, but you just missed talking about the conclusion. 3/4 of the way there.
+Academic writing - Good, but contractions pop up. 'It is' rather than 'It's'.
+Introduction does its job, but perhaps a little under-cooked. I think more could have been done here to really press the importance of the research and create a compelling case for it.
+Literature Review - A little too reliant on direct quotes. Where you have 'Lynch claims "The contents of the city images..."' He is speaking about a particular context which you then have to clarify for the reader, whereas the important part of the quote is his classification of the five types of element. You could have written this as 'Lynch (1960, pp. 46-48), in his study of images of cities, classified 5 types of physical form: paths, edges, districts, nodes, and landmarks'. Is there research you can call upon to evidence that level designers are using Lynch's research? If you say it, you need to be able to support it with evidence. I would liked to have seen a lot more research included here, and a lot more recent research. You have taken a good approach with looking at design and the 'Norman Door', but I feel more needed to be done in that opening few sections of the Lit Review to tie the concepts more tightly to level design. You do this more later on when discussing Lynch.
+Good artefact development. Ideally, to track player's data across levels, you would want to use a Game Instance class and cast to it (as it is part of the C++ engine code there is no memory overhead). The system you have implemented works for what you are doing, but were you to refine it, that would be an optimisation to consider. It would have been good to see the evolution of the project from the Grey Box environment to the finished prototype. There you could have discussed the 'Must Have' parts of the level, how you implemented and tested those in a basic set-up first before importing the final assets; and really drilled into the level design/player experience more.
+Very good discussion of the results, and you highlight with some explanation where anomalies may have occurred. A good catch that you did not ask what genre of game the two participants whose data was removed played. It may have been useful to explore more why they had issues navigating the platform stage in particular. One area that would need to be addressed is the sample size and the random split between the groups testing the artifact. Twenty is pretty low to draw data from, but you have managed to show a potential trend in the data.
+Good job, Liam. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,6 +201,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -191,7 +266,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -204,6 +279,19 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -540,16 +628,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE0FDEE9-25ED-41EF-AD75-998DC1DB7EE9}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" customWidth="1"/>
-    <col min="4" max="4" width="70.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.109375" customWidth="1"/>
+    <col min="4" max="4" width="70.109375" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.21875" style="5" customWidth="1"/>
+    <col min="8" max="8" width="11.77734375" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -562,8 +654,20 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -576,8 +680,11 @@
       <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="5">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -590,8 +697,11 @@
       <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -604,8 +714,11 @@
       <c r="D5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -618,8 +731,11 @@
       <c r="D6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="5">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -632,8 +748,11 @@
       <c r="D7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -646,8 +765,11 @@
       <c r="D8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -660,8 +782,11 @@
       <c r="D9" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="5">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -674,34 +799,68 @@
       <c r="D10" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>4</v>
+      </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="273" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="D16" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="198.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="8" t="s">
+        <v>8</v>
+      </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
+      <c r="D17" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="219" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="408.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>